<commit_message>
add placeholder for images
</commit_message>
<xml_diff>
--- a/Results.xlsx
+++ b/Results.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/filippo/Documents/GitHub_repo/Verefoo-React-Iterative---Thesis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E496192-F4BC-FC41-92BC-82472C463559}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6671C210-ED8C-1F41-861B-550214297FF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="26800" windowHeight="18000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Stanford" sheetId="1" r:id="rId1"/>
@@ -38,10 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="10">
-  <si>
-    <t>Stanford – Configuration 1   (PercentPairs: {0.5, 0.0} | PortSpecifics: 0.05)</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="17">
   <si>
     <t>Number of NSRs</t>
   </si>
@@ -50,9 +47,6 @@
   </si>
   <si>
     <t>Vanilla VEREFOO AVG [ms]</t>
-  </si>
-  <si>
-    <t>UNSAT</t>
   </si>
   <si>
     <t xml:space="preserve">CESNET </t>
@@ -67,14 +61,41 @@
     <t>Non utilizzabile causa UNSAT</t>
   </si>
   <si>
-    <t>Stanford – Configuration 2   (PercentPairs: {0.5, 0.0} | PortSpecifics: 0.3)</t>
+    <t>Run</t>
+  </si>
+  <si>
+    <t>NSR: 20</t>
+  </si>
+  <si>
+    <t>NSR: 10</t>
+  </si>
+  <si>
+    <t>NSR: 30</t>
+  </si>
+  <si>
+    <t>NSR: 40</t>
+  </si>
+  <si>
+    <t>NSR: 50</t>
+  </si>
+  <si>
+    <t>NSR: 60</t>
+  </si>
+  <si>
+    <t>Stanford  (PercentPairs: {0.5, 0.0} | PortSpecifics: 0.5)</t>
+  </si>
+  <si>
+    <t>2 UNSAT</t>
+  </si>
+  <si>
+    <t>8 UNSAT</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -108,6 +129,20 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
@@ -150,7 +185,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -201,11 +236,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFBDBDBD"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFBDBDBD"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF2C3E50"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -220,6 +268,25 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="4" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="5" fillId="4" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="5" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -340,7 +407,7 @@
                 <a:uFillTx/>
                 <a:latin typeface="Calibri"/>
               </a:rPr>
-              <a:t>Stanford – Config 2</a:t>
+              <a:t>Stanford</a:t>
             </a:r>
           </a:p>
         </c:rich>
@@ -423,7 +490,7 @@
           </c:dLbls>
           <c:cat>
             <c:numRef>
-              <c:f>Stanford!$A$13:$A$18</c:f>
+              <c:f>Stanford!$A$6:$A$11</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
@@ -450,27 +517,12 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Stanford!$B$13:$B$18</c:f>
+              <c:f>Stanford!$B$7:$B$11</c:f>
               <c:numCache>
                 <c:formatCode>#,##0.00</c:formatCode>
-                <c:ptCount val="6"/>
+                <c:ptCount val="5"/>
                 <c:pt idx="0">
-                  <c:v>103.8</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>216.05</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>353.95</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>515.95000000000005</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>711.7</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>950.45</c:v>
+                  <c:v>146321.20000000001</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -546,7 +598,7 @@
           </c:dLbls>
           <c:cat>
             <c:numRef>
-              <c:f>Stanford!$A$13:$A$18</c:f>
+              <c:f>Stanford!$A$6:$A$11</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
@@ -573,7 +625,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Stanford!$C$13:$C$18</c:f>
+              <c:f>Stanford!$C$6:$C$11</c:f>
               <c:numCache>
                 <c:formatCode>#,##0.00</c:formatCode>
                 <c:ptCount val="6"/>
@@ -1899,16 +1951,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>11880</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>76320</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>585065</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>146106</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>382680</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>111600</xdr:rowOff>
+      <xdr:colOff>292768</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>136430</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1940,16 +1992,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>175223</xdr:colOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>42701</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>189949</xdr:rowOff>
+      <xdr:rowOff>234123</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>20</xdr:col>
-      <xdr:colOff>546023</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>155971</xdr:rowOff>
+      <xdr:col>18</xdr:col>
+      <xdr:colOff>413501</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>12406</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2197,7 +2249,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:E144"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="14.5" customWidth="1"/>
@@ -2205,178 +2257,881 @@
     <col min="3" max="3" width="24.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" s="6"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+    </row>
+    <row r="4" spans="1:3" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A4" s="13" t="s">
+        <v>14</v>
+      </c>
+      <c r="B4" s="13"/>
+      <c r="C4" s="13"/>
+    </row>
+    <row r="5" spans="1:3" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-    </row>
-    <row r="2" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
+      <c r="B5" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C5" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="1" t="s">
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" s="2">
+        <v>10</v>
+      </c>
+      <c r="B6" s="8">
+        <f>AVERAGE(B15:B34)</f>
+        <v>913.15</v>
+      </c>
+      <c r="C6" s="3">
+        <v>47.25</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" s="4">
+        <v>20</v>
+      </c>
+      <c r="B7" s="8">
+        <f>AVERAGE(B37:B56)</f>
+        <v>146321.20000000001</v>
+      </c>
+      <c r="C7" s="5">
+        <v>29.15</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" s="2">
+        <v>30</v>
+      </c>
+      <c r="B8" s="8"/>
+      <c r="C8" s="3">
+        <v>69.2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" s="4">
+        <v>40</v>
+      </c>
+      <c r="B9" s="9"/>
+      <c r="C9" s="5">
+        <v>88.7</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" s="2">
+        <v>50</v>
+      </c>
+      <c r="B10" s="8"/>
+      <c r="C10" s="3">
+        <v>134.19999999999999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" s="4">
+        <v>60</v>
+      </c>
+      <c r="B11" s="9"/>
+      <c r="C11" s="5">
+        <v>209.9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="B12" s="10"/>
+    </row>
+    <row r="14" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" s="12"/>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15">
+        <v>1</v>
+      </c>
+      <c r="B15">
+        <v>2302</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16">
+        <v>2</v>
+      </c>
+      <c r="B16">
+        <v>783</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" s="2">
+      <c r="B17">
+        <v>1332</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18">
+        <v>4</v>
+      </c>
+      <c r="B18">
+        <v>2088</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19">
+        <v>5</v>
+      </c>
+      <c r="B19">
+        <v>4237</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20">
+        <v>6</v>
+      </c>
+      <c r="B20">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21">
+        <v>7</v>
+      </c>
+      <c r="B21">
+        <v>492</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22">
+        <v>8</v>
+      </c>
+      <c r="B22">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23">
+        <v>9</v>
+      </c>
+      <c r="B23">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24">
         <v>10</v>
       </c>
-      <c r="B3" s="3">
-        <v>104.9</v>
-      </c>
-      <c r="C3" s="3">
-        <v>61.1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" s="4">
+      <c r="B24">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25">
+        <v>11</v>
+      </c>
+      <c r="B25">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A26">
+        <v>12</v>
+      </c>
+      <c r="B26">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A27">
+        <v>13</v>
+      </c>
+      <c r="B27">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A28">
+        <v>14</v>
+      </c>
+      <c r="B28">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A29">
+        <v>15</v>
+      </c>
+      <c r="B29">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A30">
+        <v>16</v>
+      </c>
+      <c r="B30">
+        <v>502</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A31">
+        <v>17</v>
+      </c>
+      <c r="B31">
+        <v>893</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A32">
+        <v>18</v>
+      </c>
+      <c r="B32">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A33">
+        <v>19</v>
+      </c>
+      <c r="B33">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A34">
         <v>20</v>
       </c>
-      <c r="B4" s="5">
-        <v>218.5</v>
-      </c>
-      <c r="C4" s="5">
-        <v>44970</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" s="2">
-        <v>30</v>
-      </c>
-      <c r="B5" s="3">
-        <v>346.4</v>
-      </c>
-      <c r="C5" s="3" t="s">
+      <c r="B34">
+        <v>784</v>
+      </c>
+      <c r="E34" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B36" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C36" s="12"/>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A37">
+        <v>1</v>
+      </c>
+      <c r="B37">
+        <v>1816606</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A38">
+        <v>2</v>
+      </c>
+      <c r="B38">
+        <v>19826</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A39">
+        <v>3</v>
+      </c>
+      <c r="B39">
+        <v>251055</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A40">
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" s="4">
-        <v>40</v>
-      </c>
-      <c r="B6" s="5">
-        <v>509.3</v>
-      </c>
-      <c r="C6" s="3" t="s">
+      <c r="B40">
+        <v>18179</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A41">
+        <v>5</v>
+      </c>
+      <c r="B41">
+        <v>106233</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A42">
+        <v>6</v>
+      </c>
+      <c r="B42">
+        <v>15695</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A43">
+        <v>7</v>
+      </c>
+      <c r="B43">
+        <v>18643</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A44">
+        <v>8</v>
+      </c>
+      <c r="B44">
+        <v>30776</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A45">
+        <v>9</v>
+      </c>
+      <c r="B45">
+        <v>11636</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A46">
+        <v>10</v>
+      </c>
+      <c r="B46">
+        <v>97737</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A47">
+        <v>11</v>
+      </c>
+      <c r="B47">
+        <v>116425</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A48">
+        <v>12</v>
+      </c>
+      <c r="B48">
+        <v>104168</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A49">
+        <v>13</v>
+      </c>
+      <c r="B49">
+        <v>53539</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A50">
+        <v>14</v>
+      </c>
+      <c r="B50">
+        <v>7857</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A51">
+        <v>15</v>
+      </c>
+      <c r="B51">
+        <v>36020</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A52">
+        <v>16</v>
+      </c>
+      <c r="B52">
+        <v>22636</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A53">
+        <v>17</v>
+      </c>
+      <c r="B53">
+        <v>3276</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A54">
+        <v>18</v>
+      </c>
+      <c r="B54">
+        <v>15505</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A55">
+        <v>19</v>
+      </c>
+      <c r="B55">
+        <v>78633</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A56">
+        <v>20</v>
+      </c>
+      <c r="B56">
+        <v>101979</v>
+      </c>
+      <c r="E56" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A58" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B58" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C58" s="12"/>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A59">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A60">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A61">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A62">
         <v>4</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" s="2">
-        <v>50</v>
-      </c>
-      <c r="B7" s="3">
-        <v>648.20000000000005</v>
-      </c>
-      <c r="C7" s="3" t="s">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A63">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A64">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A65">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A66">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A67">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A68">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A69">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A70">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A71">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A72">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A73">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A74">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A75">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A76">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A77">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A78">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A80" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B80" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C80" s="12"/>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A81">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A82">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A83">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="84" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A84">
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" s="4">
-        <v>60</v>
-      </c>
-      <c r="B8" s="5">
-        <v>915.1</v>
-      </c>
-      <c r="C8" s="3" t="s">
+    <row r="85" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A85">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="86" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A86">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="87" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A87">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="88" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A88">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="89" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A89">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="90" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A90">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="91" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A91">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="92" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A92">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="93" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A93">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="94" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A94">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="95" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A95">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="96" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A96">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A97">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A98">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A99">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A100">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A102" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B102" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C102" s="12"/>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A103">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A104">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A105">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A106">
         <v>4</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="6" t="s">
+    <row r="107" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A107">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A108">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A109">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A110">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A111">
         <v>9</v>
       </c>
-      <c r="B11" s="6"/>
-      <c r="C11" s="6"/>
-    </row>
-    <row r="12" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="1" t="s">
+    </row>
+    <row r="112" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A112">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A113">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A114">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A115">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="116" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A116">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="117" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A117">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="118" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A118">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A119">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="120" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A120">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="121" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A121">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="122" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A122">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="124" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A124" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B124" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="C124" s="12"/>
+    </row>
+    <row r="125" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A125">
         <v>1</v>
       </c>
-      <c r="B12" s="1" t="s">
+    </row>
+    <row r="126" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A126">
         <v>2</v>
       </c>
-      <c r="C12" s="1" t="s">
+    </row>
+    <row r="127" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A127">
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" s="2">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A128">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="129" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A129">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="130" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A130">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="131" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A131">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="132" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A132">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="133" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A133">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="134" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A134">
         <v>10</v>
       </c>
-      <c r="B13" s="3">
-        <v>103.8</v>
-      </c>
-      <c r="C13" s="3">
-        <v>47.25</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A14" s="4">
+    </row>
+    <row r="135" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A135">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="136" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A136">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="137" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A137">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="138" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A138">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="139" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A139">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="140" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A140">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="141" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A141">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="142" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A142">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="143" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A143">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="144" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A144">
         <v>20</v>
       </c>
-      <c r="B14" s="5">
-        <v>216.05</v>
-      </c>
-      <c r="C14" s="5">
-        <v>29.15</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A15" s="2">
-        <v>30</v>
-      </c>
-      <c r="B15" s="3">
-        <v>353.95</v>
-      </c>
-      <c r="C15" s="3">
-        <v>69.2</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A16" s="4">
-        <v>40</v>
-      </c>
-      <c r="B16" s="5">
-        <v>515.95000000000005</v>
-      </c>
-      <c r="C16" s="5">
-        <v>88.7</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A17" s="2">
-        <v>50</v>
-      </c>
-      <c r="B17" s="3">
-        <v>711.7</v>
-      </c>
-      <c r="C17" s="3">
-        <v>134.19999999999999</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A18" s="4">
-        <v>60</v>
-      </c>
-      <c r="B18" s="5">
-        <v>950.45</v>
-      </c>
-      <c r="C18" s="5">
-        <v>209.9</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A11:C11"/>
+  <mergeCells count="7">
+    <mergeCell ref="B58:C58"/>
+    <mergeCell ref="B80:C80"/>
+    <mergeCell ref="B102:C102"/>
+    <mergeCell ref="B124:C124"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B36:C36"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -2396,25 +3151,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="7" t="s">
-        <v>5</v>
-      </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
+      <c r="A1" s="14" t="s">
+        <v>3</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
+      <c r="D1" s="14"/>
     </row>
     <row r="2" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>2</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.2">
@@ -2424,7 +3179,7 @@
       <c r="B3" s="2">
         <v>20</v>
       </c>
-      <c r="C3" s="3">
+      <c r="C3" s="8">
         <f>AVERAGE(C12:C31)</f>
         <v>345.7</v>
       </c>
@@ -2440,7 +3195,7 @@
       <c r="B4" s="4">
         <v>40</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="9">
         <f>AVERAGE(C33:C52)</f>
         <v>670.4</v>
       </c>
@@ -2456,7 +3211,7 @@
       <c r="B5" s="2">
         <v>60</v>
       </c>
-      <c r="C5" s="3">
+      <c r="C5" s="8">
         <f>AVERAGE(C54:C73)</f>
         <v>975.15</v>
       </c>
@@ -2472,7 +3227,7 @@
       <c r="B6" s="4">
         <v>80</v>
       </c>
-      <c r="C6" s="5">
+      <c r="C6" s="9">
         <f>AVERAGE(C75:C96)</f>
         <v>1302.047619047619</v>
       </c>
@@ -2488,7 +3243,7 @@
       <c r="B7" s="2">
         <v>100</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7" s="8">
         <f>AVERAGE(C96:C115)</f>
         <v>1587.3</v>
       </c>
@@ -2504,7 +3259,7 @@
       <c r="B8" s="4">
         <v>120</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C8" s="9">
         <f>AVERAGE(C117:C136)</f>
         <v>1912.1</v>
       </c>
@@ -2513,7 +3268,7 @@
         <v>966891.85</v>
       </c>
       <c r="F8" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
@@ -3517,28 +4272,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
+      <c r="A1" s="14" t="s">
+        <v>5</v>
+      </c>
+      <c r="B1" s="14"/>
+      <c r="C1" s="14"/>
     </row>
     <row r="2" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>2</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
         <v>48</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="8">
         <v>514</v>
       </c>
       <c r="C3" s="3">
@@ -3549,7 +4304,7 @@
       <c r="A4" s="4">
         <v>96</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="9">
         <v>1453</v>
       </c>
       <c r="C4" s="5">
@@ -3560,7 +4315,7 @@
       <c r="A5" s="2">
         <v>144</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="8">
         <v>3765</v>
       </c>
       <c r="C5" s="3">
@@ -3571,7 +4326,7 @@
       <c r="A6" s="4">
         <v>192</v>
       </c>
-      <c r="B6" s="5">
+      <c r="B6" s="9">
         <v>5970</v>
       </c>
       <c r="C6" s="5">
@@ -3582,7 +4337,7 @@
       <c r="A7" s="2">
         <v>240</v>
       </c>
-      <c r="B7" s="3">
+      <c r="B7" s="8">
         <v>10922</v>
       </c>
       <c r="C7" s="3">
@@ -3593,7 +4348,7 @@
       <c r="A8" s="4">
         <v>288</v>
       </c>
-      <c r="B8" s="5">
+      <c r="B8" s="9">
         <v>17083</v>
       </c>
       <c r="C8" s="5">

</xml_diff>

<commit_message>
aligned version with Serializer on VM + cosmetical on thesis
</commit_message>
<xml_diff>
--- a/Results.xlsx
+++ b/Results.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10719"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10821"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/filippo/Documents/GitHub_repo/Verefoo-React-Iterative---Thesis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6671C210-ED8C-1F41-861B-550214297FF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E06AC04A-1190-084B-BA8A-08988BB3DE9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="25820" windowHeight="18000" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Stanford" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="28">
   <si>
     <t>Number of NSRs</t>
   </si>
@@ -47,9 +47,6 @@
   </si>
   <si>
     <t>Vanilla VEREFOO AVG [ms]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">CESNET </t>
   </si>
   <si>
     <t>PolicyNumber</t>
@@ -89,6 +86,42 @@
   </si>
   <si>
     <t>8 UNSAT</t>
+  </si>
+  <si>
+    <t>ReachPerc</t>
+  </si>
+  <si>
+    <t>0.5</t>
+  </si>
+  <si>
+    <t>0.48</t>
+  </si>
+  <si>
+    <t>0.51</t>
+  </si>
+  <si>
+    <t>0.49</t>
+  </si>
+  <si>
+    <t>1, 3</t>
+  </si>
+  <si>
+    <t>2, 6</t>
+  </si>
+  <si>
+    <t>3, 9</t>
+  </si>
+  <si>
+    <t>4, 12</t>
+  </si>
+  <si>
+    <t>5, 15</t>
+  </si>
+  <si>
+    <t>6, 18</t>
+  </si>
+  <si>
+    <t>CESNET; Reacheability Percenteage always around 0.5</t>
   </si>
 </sst>
 </file>
@@ -1004,7 +1037,7 @@
           </c:dLbls>
           <c:cat>
             <c:numRef>
-              <c:f>CESNET!$B$3:$B$8</c:f>
+              <c:f>CESNET!$C$3:$C$8</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
@@ -1031,7 +1064,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>CESNET!$C$3:$C$8</c:f>
+              <c:f>CESNET!$D$3:$D$8</c:f>
               <c:numCache>
                 <c:formatCode>#,##0.00</c:formatCode>
                 <c:ptCount val="6"/>
@@ -1132,7 +1165,7 @@
           </c:dLbls>
           <c:cat>
             <c:numRef>
-              <c:f>CESNET!$B$3:$B$8</c:f>
+              <c:f>CESNET!$C$3:$C$8</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
@@ -1159,7 +1192,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>CESNET!$D$3:$D$8</c:f>
+              <c:f>CESNET!$E$3:$E$8</c:f>
               <c:numCache>
                 <c:formatCode>#,##0.00</c:formatCode>
                 <c:ptCount val="6"/>
@@ -1533,7 +1566,7 @@
           </c:dLbls>
           <c:cat>
             <c:numRef>
-              <c:f>Texas2000!$A$3:$A$8</c:f>
+              <c:f>Texas2000!$B$3:$B$8</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
@@ -1560,7 +1593,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Texas2000!$B$3:$B$8</c:f>
+              <c:f>Texas2000!$C$3:$C$8</c:f>
               <c:numCache>
                 <c:formatCode>#,##0.00</c:formatCode>
                 <c:ptCount val="6"/>
@@ -1656,7 +1689,7 @@
           </c:dLbls>
           <c:cat>
             <c:numRef>
-              <c:f>Texas2000!$A$3:$A$8</c:f>
+              <c:f>Texas2000!$B$3:$B$8</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="6"/>
@@ -1683,7 +1716,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Texas2000!$C$3:$C$8</c:f>
+              <c:f>Texas2000!$D$3:$D$8</c:f>
               <c:numCache>
                 <c:formatCode>#,##0.00</c:formatCode>
                 <c:ptCount val="6"/>
@@ -1952,15 +1985,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>585065</xdr:colOff>
+      <xdr:colOff>438959</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>146106</xdr:rowOff>
+      <xdr:rowOff>168584</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>14</xdr:col>
-      <xdr:colOff>292768</xdr:colOff>
+      <xdr:colOff>146662</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>136430</xdr:rowOff>
+      <xdr:rowOff>158908</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -1992,13 +2025,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>8</xdr:col>
+      <xdr:col>9</xdr:col>
       <xdr:colOff>42701</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>234123</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>18</xdr:col>
+      <xdr:col>19</xdr:col>
       <xdr:colOff>413501</xdr:colOff>
       <xdr:row>23</xdr:row>
       <xdr:rowOff>12406</xdr:rowOff>
@@ -2033,14 +2066,14 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>4</xdr:col>
+      <xdr:col>5</xdr:col>
       <xdr:colOff>118440</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>101520</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>488880</xdr:colOff>
+      <xdr:col>15</xdr:col>
+      <xdr:colOff>488879</xdr:colOff>
       <xdr:row>22</xdr:row>
       <xdr:rowOff>68040</xdr:rowOff>
     </xdr:to>
@@ -2264,7 +2297,7 @@
     </row>
     <row r="4" spans="1:3" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="13" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B4" s="13"/>
       <c r="C4" s="13"/>
@@ -2345,10 +2378,10 @@
     </row>
     <row r="14" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C14" s="12"/>
     </row>
@@ -2512,15 +2545,15 @@
         <v>784</v>
       </c>
       <c r="E34" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="36" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B36" s="11" t="s">
         <v>7</v>
-      </c>
-      <c r="B36" s="11" t="s">
-        <v>8</v>
       </c>
       <c r="C36" s="12"/>
     </row>
@@ -2684,15 +2717,15 @@
         <v>101979</v>
       </c>
       <c r="E56" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
     </row>
     <row r="58" spans="1:5" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B58" s="11" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C58" s="12"/>
     </row>
@@ -2798,10 +2831,10 @@
     </row>
     <row r="80" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A80" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B80" s="11" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C80" s="12"/>
     </row>
@@ -2907,10 +2940,10 @@
     </row>
     <row r="102" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A102" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B102" s="11" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C102" s="12"/>
     </row>
@@ -3016,10 +3049,10 @@
     </row>
     <row r="124" spans="1:3" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A124" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B124" s="11" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C124" s="12"/>
     </row>
@@ -3141,1122 +3174,1144 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:F136"/>
+  <dimension ref="A1:G136"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="12.6640625" customWidth="1"/>
-    <col min="2" max="2" width="14.5" customWidth="1"/>
-    <col min="3" max="3" width="21.5" customWidth="1"/>
-    <col min="4" max="4" width="24.1640625" customWidth="1"/>
+    <col min="1" max="2" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="14.5" customWidth="1"/>
+    <col min="4" max="4" width="21.5" customWidth="1"/>
+    <col min="5" max="5" width="24.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="14" t="s">
-        <v>3</v>
+        <v>27</v>
       </c>
       <c r="B1" s="14"/>
       <c r="C1" s="14"/>
       <c r="D1" s="14"/>
-    </row>
-    <row r="2" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="E1" s="14"/>
+    </row>
+    <row r="2" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
         <v>13</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" s="2">
         <v>20</v>
       </c>
-      <c r="C3" s="8">
-        <f>AVERAGE(C12:C31)</f>
+      <c r="D3" s="8">
+        <f>AVERAGE(D12:D31)</f>
         <v>345.7</v>
       </c>
-      <c r="D3" s="3">
-        <f>AVERAGE(D12:D31)</f>
+      <c r="E3" s="3">
+        <f>AVERAGE(E12:E31)</f>
         <v>2540.75</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A4" s="4">
         <v>27</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" s="4">
         <v>40</v>
       </c>
-      <c r="C4" s="9">
-        <f>AVERAGE(C33:C52)</f>
+      <c r="D4" s="9">
+        <f>AVERAGE(D33:D52)</f>
         <v>670.4</v>
       </c>
-      <c r="D4" s="5">
-        <f>AVERAGE(D33:D52)</f>
+      <c r="E4" s="5">
+        <f>AVERAGE(E33:E52)</f>
         <v>15034.1</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
         <v>40</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="C5" s="2">
         <v>60</v>
       </c>
-      <c r="C5" s="8">
-        <f>AVERAGE(C54:C73)</f>
+      <c r="D5" s="8">
+        <f>AVERAGE(D54:D73)</f>
         <v>975.15</v>
       </c>
-      <c r="D5" s="3">
-        <f>AVERAGE(D54:D73)</f>
+      <c r="E5" s="3">
+        <f>AVERAGE(E54:E73)</f>
         <v>43808.9</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A6" s="4">
         <v>53</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B6" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C6" s="4">
         <v>80</v>
       </c>
-      <c r="C6" s="9">
-        <f>AVERAGE(C75:C96)</f>
+      <c r="D6" s="9">
+        <f>AVERAGE(D75:D96)</f>
         <v>1302.047619047619</v>
       </c>
-      <c r="D6" s="5">
-        <f>AVERAGE(D75:D96)</f>
+      <c r="E6" s="5">
+        <f>AVERAGE(E75:E96)</f>
         <v>124081.90476190476</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
         <v>67</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="2">
         <v>100</v>
       </c>
-      <c r="C7" s="8">
-        <f>AVERAGE(C96:C115)</f>
+      <c r="D7" s="8">
+        <f>AVERAGE(D96:D115)</f>
         <v>1587.3</v>
       </c>
-      <c r="D7" s="3">
-        <f>AVERAGE(D96:D115)</f>
+      <c r="E7" s="3">
+        <f>AVERAGE(E96:E115)</f>
         <v>356093.25</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A8" s="4">
         <v>80</v>
       </c>
-      <c r="B8" s="4">
+      <c r="B8" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" s="4">
         <v>120</v>
       </c>
-      <c r="C8" s="9">
-        <f>AVERAGE(C117:C136)</f>
+      <c r="D8" s="9">
+        <f>AVERAGE(D117:D136)</f>
         <v>1912.1</v>
       </c>
-      <c r="D8" s="5">
-        <f>AVERAGE(D117:D136)</f>
+      <c r="E8" s="5">
+        <f>AVERAGE(E117:E136)</f>
         <v>966891.85</v>
       </c>
-      <c r="F8" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="B12">
+      <c r="G8" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="C12">
         <v>20</v>
       </c>
-      <c r="C12">
+      <c r="D12">
         <v>519</v>
       </c>
-      <c r="D12">
+      <c r="E12">
         <v>1530</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="C13">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="D13">
         <v>310</v>
       </c>
-      <c r="D13">
+      <c r="E13">
         <v>3312</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="C14">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="D14">
         <v>270</v>
       </c>
-      <c r="D14">
+      <c r="E14">
         <v>1532</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="C15">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="D15">
         <v>303</v>
       </c>
-      <c r="D15">
+      <c r="E15">
         <v>1598</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="C16">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="D16">
         <v>324</v>
       </c>
-      <c r="D16">
+      <c r="E16">
         <v>2765</v>
       </c>
     </row>
-    <row r="17" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C17">
+    <row r="17" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D17">
         <v>506</v>
       </c>
-      <c r="D17">
+      <c r="E17">
         <v>2191</v>
       </c>
     </row>
-    <row r="18" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C18">
+    <row r="18" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D18">
         <v>324</v>
       </c>
-      <c r="D18">
+      <c r="E18">
         <v>2724</v>
       </c>
     </row>
-    <row r="19" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C19">
+    <row r="19" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D19">
         <v>311</v>
       </c>
-      <c r="D19">
+      <c r="E19">
         <v>1089</v>
       </c>
     </row>
-    <row r="20" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C20">
+    <row r="20" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D20">
         <v>288</v>
       </c>
-      <c r="D20">
+      <c r="E20">
         <v>3007</v>
       </c>
     </row>
-    <row r="21" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C21">
+    <row r="21" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D21">
         <v>298</v>
       </c>
-      <c r="D21">
+      <c r="E21">
         <v>3599</v>
       </c>
     </row>
-    <row r="22" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C22">
+    <row r="22" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D22">
         <v>477</v>
       </c>
-      <c r="D22">
+      <c r="E22">
         <v>2722</v>
       </c>
     </row>
-    <row r="23" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C23">
+    <row r="23" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D23">
         <v>337</v>
       </c>
-      <c r="D23">
+      <c r="E23">
         <v>3208</v>
       </c>
     </row>
-    <row r="24" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C24">
+    <row r="24" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D24">
         <v>316</v>
       </c>
-      <c r="D24">
+      <c r="E24">
         <v>3274</v>
       </c>
     </row>
-    <row r="25" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C25">
+    <row r="25" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D25">
         <v>300</v>
       </c>
-      <c r="D25">
+      <c r="E25">
         <v>1498</v>
       </c>
     </row>
-    <row r="26" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C26">
+    <row r="26" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D26">
         <v>336</v>
       </c>
-      <c r="D26">
+      <c r="E26">
         <v>3968</v>
       </c>
     </row>
-    <row r="27" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C27">
+    <row r="27" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D27">
         <v>484</v>
       </c>
-      <c r="D27">
+      <c r="E27">
         <v>1237</v>
       </c>
     </row>
-    <row r="28" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C28">
+    <row r="28" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D28">
         <v>326</v>
       </c>
-      <c r="D28">
+      <c r="E28">
         <v>2341</v>
       </c>
     </row>
-    <row r="29" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C29">
+    <row r="29" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D29">
         <v>292</v>
       </c>
-      <c r="D29">
+      <c r="E29">
         <v>3213</v>
       </c>
     </row>
-    <row r="30" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C30">
+    <row r="30" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D30">
         <v>324</v>
       </c>
-      <c r="D30">
+      <c r="E30">
         <v>3438</v>
       </c>
     </row>
-    <row r="31" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C31">
+    <row r="31" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D31">
         <v>269</v>
       </c>
-      <c r="D31">
+      <c r="E31">
         <v>2569</v>
       </c>
     </row>
-    <row r="33" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B33">
+    <row r="33" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C33">
         <v>40</v>
       </c>
-      <c r="C33">
+      <c r="D33">
         <v>825</v>
       </c>
-      <c r="D33">
+      <c r="E33">
         <v>27677</v>
       </c>
     </row>
-    <row r="34" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C34">
+    <row r="34" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D34">
         <v>592</v>
       </c>
-      <c r="D34">
+      <c r="E34">
         <v>18611</v>
       </c>
     </row>
-    <row r="35" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C35">
+    <row r="35" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D35">
         <v>660</v>
       </c>
-      <c r="D35">
+      <c r="E35">
         <v>14865</v>
       </c>
     </row>
-    <row r="36" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C36">
+    <row r="36" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D36">
         <v>594</v>
       </c>
-      <c r="D36">
+      <c r="E36">
         <v>16031</v>
       </c>
     </row>
-    <row r="37" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C37">
+    <row r="37" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D37">
         <v>589</v>
       </c>
-      <c r="D37">
+      <c r="E37">
         <v>14320</v>
       </c>
     </row>
-    <row r="38" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C38">
+    <row r="38" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D38">
         <v>890</v>
       </c>
-      <c r="D38">
+      <c r="E38">
         <v>18178</v>
       </c>
     </row>
-    <row r="39" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C39">
+    <row r="39" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D39">
         <v>671</v>
       </c>
-      <c r="D39">
+      <c r="E39">
         <v>17974</v>
       </c>
     </row>
-    <row r="40" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C40">
+    <row r="40" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D40">
         <v>624</v>
       </c>
-      <c r="D40">
+      <c r="E40">
         <v>10397</v>
       </c>
     </row>
-    <row r="41" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C41">
+    <row r="41" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D41">
         <v>610</v>
       </c>
-      <c r="D41">
+      <c r="E41">
         <v>15896</v>
       </c>
     </row>
-    <row r="42" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C42">
+    <row r="42" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D42">
         <v>603</v>
       </c>
-      <c r="D42">
+      <c r="E42">
         <v>16493</v>
       </c>
     </row>
-    <row r="43" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C43">
+    <row r="43" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D43">
         <v>846</v>
       </c>
-      <c r="D43">
+      <c r="E43">
         <v>10689</v>
       </c>
     </row>
-    <row r="44" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C44">
+    <row r="44" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D44">
         <v>652</v>
       </c>
-      <c r="D44">
+      <c r="E44">
         <v>8260</v>
       </c>
     </row>
-    <row r="45" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C45">
+    <row r="45" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D45">
         <v>573</v>
       </c>
-      <c r="D45">
+      <c r="E45">
         <v>14787</v>
       </c>
     </row>
-    <row r="46" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C46">
+    <row r="46" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D46">
         <v>650</v>
       </c>
-      <c r="D46">
+      <c r="E46">
         <v>18125</v>
       </c>
     </row>
-    <row r="47" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C47">
+    <row r="47" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D47">
         <v>619</v>
       </c>
-      <c r="D47">
+      <c r="E47">
         <v>17589</v>
       </c>
     </row>
-    <row r="48" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C48">
+    <row r="48" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D48">
         <v>859</v>
       </c>
-      <c r="D48">
+      <c r="E48">
         <v>11251</v>
       </c>
     </row>
-    <row r="49" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C49">
+    <row r="49" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D49">
         <v>615</v>
       </c>
-      <c r="D49">
+      <c r="E49">
         <v>10239</v>
       </c>
     </row>
-    <row r="50" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C50">
+    <row r="50" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D50">
         <v>672</v>
       </c>
-      <c r="D50">
+      <c r="E50">
         <v>14143</v>
       </c>
     </row>
-    <row r="51" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C51">
+    <row r="51" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D51">
         <v>628</v>
       </c>
-      <c r="D51">
+      <c r="E51">
         <v>13193</v>
       </c>
     </row>
-    <row r="52" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C52">
+    <row r="52" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D52">
         <v>636</v>
       </c>
-      <c r="D52">
+      <c r="E52">
         <v>11964</v>
       </c>
     </row>
-    <row r="54" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B54">
+    <row r="54" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C54">
         <v>60</v>
       </c>
-      <c r="C54">
+      <c r="D54">
         <v>1122</v>
       </c>
-      <c r="D54">
+      <c r="E54">
         <v>44209</v>
       </c>
     </row>
-    <row r="55" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C55">
+    <row r="55" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D55">
         <v>989</v>
       </c>
-      <c r="D55">
+      <c r="E55">
         <v>35543</v>
       </c>
     </row>
-    <row r="56" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C56">
+    <row r="56" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D56">
         <v>1003</v>
       </c>
-      <c r="D56">
+      <c r="E56">
         <v>57657</v>
       </c>
     </row>
-    <row r="57" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C57">
+    <row r="57" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D57">
         <v>911</v>
       </c>
-      <c r="D57">
+      <c r="E57">
         <v>19411</v>
       </c>
     </row>
-    <row r="58" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C58">
+    <row r="58" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D58">
         <v>872</v>
       </c>
-      <c r="D58">
+      <c r="E58">
         <v>34554</v>
       </c>
     </row>
-    <row r="59" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C59">
+    <row r="59" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D59">
         <v>1143</v>
       </c>
-      <c r="D59">
+      <c r="E59">
         <v>24369</v>
       </c>
     </row>
-    <row r="60" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C60">
+    <row r="60" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D60">
         <v>1026</v>
       </c>
-      <c r="D60">
+      <c r="E60">
         <v>43924</v>
       </c>
     </row>
-    <row r="61" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C61">
+    <row r="61" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D61">
         <v>922</v>
       </c>
-      <c r="D61">
+      <c r="E61">
         <v>53228</v>
       </c>
     </row>
-    <row r="62" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C62">
+    <row r="62" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D62">
         <v>922</v>
       </c>
-      <c r="D62">
+      <c r="E62">
         <v>39917</v>
       </c>
     </row>
-    <row r="63" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C63">
+    <row r="63" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D63">
         <v>857</v>
       </c>
-      <c r="D63">
+      <c r="E63">
         <v>30242</v>
       </c>
     </row>
-    <row r="64" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C64">
+    <row r="64" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D64">
         <v>1177</v>
       </c>
-      <c r="D64">
+      <c r="E64">
         <v>67379</v>
       </c>
     </row>
-    <row r="65" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C65">
+    <row r="65" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D65">
         <v>967</v>
       </c>
-      <c r="D65">
+      <c r="E65">
         <v>38393</v>
       </c>
     </row>
-    <row r="66" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C66">
+    <row r="66" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D66">
         <v>891</v>
       </c>
-      <c r="D66">
+      <c r="E66">
         <v>66375</v>
       </c>
     </row>
-    <row r="67" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C67">
+    <row r="67" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D67">
         <v>935</v>
       </c>
-      <c r="D67">
+      <c r="E67">
         <v>24403</v>
       </c>
     </row>
-    <row r="68" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C68">
+    <row r="68" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D68">
         <v>926</v>
       </c>
-      <c r="D68">
+      <c r="E68">
         <v>29486</v>
       </c>
     </row>
-    <row r="69" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C69">
+    <row r="69" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D69">
         <v>1145</v>
       </c>
-      <c r="D69">
+      <c r="E69">
         <v>59560</v>
       </c>
     </row>
-    <row r="70" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C70">
+    <row r="70" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D70">
         <v>963</v>
       </c>
-      <c r="D70">
+      <c r="E70">
         <v>44514</v>
       </c>
     </row>
-    <row r="71" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C71">
+    <row r="71" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D71">
         <v>988</v>
       </c>
-      <c r="D71">
+      <c r="E71">
         <v>47679</v>
       </c>
     </row>
-    <row r="72" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C72">
+    <row r="72" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D72">
         <v>878</v>
       </c>
-      <c r="D72">
+      <c r="E72">
         <v>61758</v>
       </c>
     </row>
-    <row r="73" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C73">
+    <row r="73" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D73">
         <v>866</v>
       </c>
-      <c r="D73">
+      <c r="E73">
         <v>53577</v>
       </c>
     </row>
-    <row r="75" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B75">
+    <row r="75" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C75">
         <v>80</v>
       </c>
-      <c r="C75">
+      <c r="D75">
         <v>1514</v>
       </c>
-      <c r="D75">
+      <c r="E75">
         <v>111842</v>
       </c>
     </row>
-    <row r="76" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C76">
+    <row r="76" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D76">
         <v>1227</v>
       </c>
-      <c r="D76">
+      <c r="E76">
         <v>97396</v>
       </c>
     </row>
-    <row r="77" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C77">
+    <row r="77" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D77">
         <v>1193</v>
       </c>
-      <c r="D77">
+      <c r="E77">
         <v>67459</v>
       </c>
     </row>
-    <row r="78" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C78">
+    <row r="78" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D78">
         <v>1285</v>
       </c>
-      <c r="D78">
+      <c r="E78">
         <v>106312</v>
       </c>
     </row>
-    <row r="79" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C79">
+    <row r="79" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D79">
         <v>1200</v>
       </c>
-      <c r="D79">
+      <c r="E79">
         <v>187055</v>
       </c>
     </row>
-    <row r="80" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C80">
+    <row r="80" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D80">
         <v>1477</v>
       </c>
-      <c r="D80">
+      <c r="E80">
         <v>6561</v>
       </c>
     </row>
-    <row r="81" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C81">
+    <row r="81" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D81">
         <v>1295</v>
       </c>
-      <c r="D81">
+      <c r="E81">
         <v>134749</v>
       </c>
     </row>
-    <row r="82" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C82">
+    <row r="82" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D82">
         <v>1225</v>
       </c>
-      <c r="D82">
+      <c r="E82">
         <v>137259</v>
       </c>
     </row>
-    <row r="83" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C83">
+    <row r="83" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D83">
         <v>1222</v>
       </c>
-      <c r="D83">
+      <c r="E83">
         <v>187679</v>
       </c>
     </row>
-    <row r="84" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C84">
+    <row r="84" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D84">
         <v>1186</v>
       </c>
-      <c r="D84">
+      <c r="E84">
         <v>129964</v>
       </c>
     </row>
-    <row r="85" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C85">
+    <row r="85" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D85">
         <v>1444</v>
       </c>
-      <c r="D85">
+      <c r="E85">
         <v>118073</v>
       </c>
     </row>
-    <row r="86" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C86">
+    <row r="86" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D86">
         <v>1208</v>
       </c>
-      <c r="D86">
+      <c r="E86">
         <v>148009</v>
       </c>
     </row>
-    <row r="87" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C87">
+    <row r="87" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D87">
         <v>1228</v>
       </c>
-      <c r="D87">
+      <c r="E87">
         <v>104379</v>
       </c>
     </row>
-    <row r="88" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C88">
+    <row r="88" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D88">
         <v>1204</v>
       </c>
-      <c r="D88">
+      <c r="E88">
         <v>87577</v>
       </c>
     </row>
-    <row r="89" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C89">
+    <row r="89" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D89">
         <v>1223</v>
       </c>
-      <c r="D89">
+      <c r="E89">
         <v>97216</v>
       </c>
     </row>
-    <row r="90" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C90">
+    <row r="90" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D90">
         <v>1450</v>
       </c>
-      <c r="D90">
+      <c r="E90">
         <v>81893</v>
       </c>
     </row>
-    <row r="91" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C91">
+    <row r="91" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D91">
         <v>1268</v>
       </c>
-      <c r="D91">
+      <c r="E91">
         <v>141358</v>
       </c>
     </row>
-    <row r="92" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C92">
+    <row r="92" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D92">
         <v>1190</v>
       </c>
-      <c r="D92">
+      <c r="E92">
         <v>76260</v>
       </c>
     </row>
-    <row r="93" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C93">
+    <row r="93" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D93">
         <v>1257</v>
       </c>
-      <c r="D93">
+      <c r="E93">
         <v>208572</v>
       </c>
     </row>
-    <row r="94" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C94">
+    <row r="94" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D94">
         <v>1240</v>
       </c>
-      <c r="D94">
+      <c r="E94">
         <v>130635</v>
       </c>
     </row>
-    <row r="96" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B96">
+    <row r="96" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C96">
         <v>100</v>
       </c>
-      <c r="C96">
+      <c r="D96">
         <v>1807</v>
       </c>
-      <c r="D96">
+      <c r="E96">
         <v>245472</v>
       </c>
     </row>
-    <row r="97" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C97">
+    <row r="97" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D97">
         <v>1627</v>
       </c>
-      <c r="D97">
+      <c r="E97">
         <v>345978</v>
       </c>
     </row>
-    <row r="98" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C98">
+    <row r="98" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D98">
         <v>1517</v>
       </c>
-      <c r="D98">
+      <c r="E98">
         <v>77058</v>
       </c>
     </row>
-    <row r="99" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C99">
+    <row r="99" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D99">
         <v>1471</v>
       </c>
-      <c r="D99">
+      <c r="E99">
         <v>272895</v>
       </c>
     </row>
-    <row r="100" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C100">
+    <row r="100" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D100">
         <v>1489</v>
       </c>
-      <c r="D100">
+      <c r="E100">
         <v>363581</v>
       </c>
     </row>
-    <row r="101" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C101">
+    <row r="101" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D101">
         <v>1852</v>
       </c>
-      <c r="D101">
+      <c r="E101">
         <v>355934</v>
       </c>
     </row>
-    <row r="102" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C102">
+    <row r="102" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D102">
         <v>1552</v>
       </c>
-      <c r="D102">
+      <c r="E102">
         <v>204211</v>
       </c>
     </row>
-    <row r="103" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C103">
+    <row r="103" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D103">
         <v>1453</v>
       </c>
-      <c r="D103">
+      <c r="E103">
         <v>163761</v>
       </c>
     </row>
-    <row r="104" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C104">
+    <row r="104" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D104">
         <v>1544</v>
       </c>
-      <c r="D104">
+      <c r="E104">
         <v>355336</v>
       </c>
     </row>
-    <row r="105" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C105">
+    <row r="105" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D105">
         <v>1490</v>
       </c>
-      <c r="D105">
+      <c r="E105">
         <v>242422</v>
       </c>
     </row>
-    <row r="106" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C106">
+    <row r="106" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D106">
         <v>1751</v>
       </c>
-      <c r="D106">
+      <c r="E106">
         <v>336964</v>
       </c>
     </row>
-    <row r="107" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C107">
+    <row r="107" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D107">
         <v>1592</v>
       </c>
-      <c r="D107">
+      <c r="E107">
         <v>731159</v>
       </c>
     </row>
-    <row r="108" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C108">
+    <row r="108" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D108">
         <v>1548</v>
       </c>
-      <c r="D108">
+      <c r="E108">
         <v>784391</v>
       </c>
     </row>
-    <row r="109" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C109">
+    <row r="109" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D109">
         <v>1529</v>
       </c>
-      <c r="D109">
+      <c r="E109">
         <v>457760</v>
       </c>
     </row>
-    <row r="110" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C110">
+    <row r="110" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D110">
         <v>1448</v>
       </c>
-      <c r="D110">
+      <c r="E110">
         <v>347017</v>
       </c>
     </row>
-    <row r="111" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C111">
+    <row r="111" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D111">
         <v>1871</v>
       </c>
-      <c r="D111">
+      <c r="E111">
         <v>367808</v>
       </c>
     </row>
-    <row r="112" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C112">
+    <row r="112" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D112">
         <v>1599</v>
       </c>
-      <c r="D112">
+      <c r="E112">
         <v>323543</v>
       </c>
     </row>
-    <row r="113" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C113">
+    <row r="113" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D113">
         <v>1596</v>
       </c>
-      <c r="D113">
+      <c r="E113">
         <v>749379</v>
       </c>
     </row>
-    <row r="114" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C114">
+    <row r="114" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D114">
         <v>1539</v>
       </c>
-      <c r="D114">
+      <c r="E114">
         <v>82293</v>
       </c>
     </row>
-    <row r="115" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C115">
+    <row r="115" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D115">
         <v>1471</v>
       </c>
-      <c r="D115">
+      <c r="E115">
         <v>314903</v>
       </c>
     </row>
-    <row r="117" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B117">
+    <row r="117" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="C117">
         <v>120</v>
       </c>
-      <c r="C117">
+      <c r="D117">
         <v>2154</v>
       </c>
-      <c r="D117">
+      <c r="E117">
         <v>511798</v>
       </c>
     </row>
-    <row r="118" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C118">
+    <row r="118" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D118">
         <v>1977</v>
       </c>
-      <c r="D118">
+      <c r="E118">
         <v>1813172</v>
       </c>
     </row>
-    <row r="119" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C119">
+    <row r="119" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D119">
         <v>1804</v>
       </c>
-      <c r="D119">
+      <c r="E119">
         <v>1815678</v>
       </c>
     </row>
-    <row r="120" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C120">
+    <row r="120" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D120">
         <v>1780</v>
       </c>
-      <c r="D120">
+      <c r="E120">
         <v>319548</v>
       </c>
     </row>
-    <row r="121" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C121">
+    <row r="121" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D121">
         <v>1760</v>
       </c>
-      <c r="D121">
+      <c r="E121">
         <v>281338</v>
       </c>
     </row>
-    <row r="122" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C122">
+    <row r="122" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D122">
         <v>2217</v>
       </c>
-      <c r="D122">
+      <c r="E122">
         <v>1810140</v>
       </c>
     </row>
-    <row r="123" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C123">
+    <row r="123" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D123">
         <v>1968</v>
       </c>
-      <c r="D123">
+      <c r="E123">
         <v>689513</v>
       </c>
     </row>
-    <row r="124" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C124">
+    <row r="124" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D124">
         <v>1882</v>
       </c>
-      <c r="D124">
+      <c r="E124">
         <v>1812181</v>
       </c>
     </row>
-    <row r="125" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C125">
+    <row r="125" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D125">
         <v>1811</v>
       </c>
-      <c r="D125">
+      <c r="E125">
         <v>413289</v>
       </c>
     </row>
-    <row r="126" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C126">
+    <row r="126" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D126">
         <v>1829</v>
       </c>
-      <c r="D126">
+      <c r="E126">
         <v>422554</v>
       </c>
     </row>
-    <row r="127" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C127">
+    <row r="127" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D127">
         <v>2160</v>
       </c>
-      <c r="D127">
+      <c r="E127">
         <v>1811122</v>
       </c>
     </row>
-    <row r="128" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="C128">
+    <row r="128" spans="3:5" x14ac:dyDescent="0.2">
+      <c r="D128">
         <v>1866</v>
       </c>
-      <c r="D128">
+      <c r="E128">
         <v>366224</v>
       </c>
     </row>
-    <row r="129" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C129">
+    <row r="129" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D129">
         <v>1853</v>
       </c>
-      <c r="D129">
+      <c r="E129">
         <v>1810420</v>
       </c>
     </row>
-    <row r="130" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C130">
+    <row r="130" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D130">
         <v>1867</v>
       </c>
-      <c r="D130">
+      <c r="E130">
         <v>382995</v>
       </c>
     </row>
-    <row r="131" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C131">
+    <row r="131" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D131">
         <v>1814</v>
       </c>
-      <c r="D131">
+      <c r="E131">
         <v>12985</v>
       </c>
     </row>
-    <row r="132" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C132">
+    <row r="132" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D132">
         <v>2221</v>
       </c>
-      <c r="D132">
+      <c r="E132">
         <v>490208</v>
       </c>
     </row>
-    <row r="133" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C133">
+    <row r="133" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D133">
         <v>1809</v>
       </c>
-      <c r="D133">
+      <c r="E133">
         <v>268306</v>
       </c>
     </row>
-    <row r="134" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C134">
+    <row r="134" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D134">
         <v>1888</v>
       </c>
-      <c r="D134">
+      <c r="E134">
         <v>682238</v>
       </c>
     </row>
-    <row r="135" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C135">
+    <row r="135" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D135">
         <v>1824</v>
       </c>
-      <c r="D135">
+      <c r="E135">
         <v>1812568</v>
       </c>
     </row>
-    <row r="136" spans="3:4" x14ac:dyDescent="0.2">
-      <c r="C136">
+    <row r="136" spans="4:5" x14ac:dyDescent="0.2">
+      <c r="D136">
         <v>1758</v>
       </c>
-      <c r="D136">
+      <c r="E136">
         <v>1811560</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A1:E1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
   <ignoredErrors>
-    <ignoredError sqref="D6" formulaRange="1"/>
+    <ignoredError sqref="E6" formulaRange="1"/>
   </ignoredErrors>
   <drawing r:id="rId1"/>
 </worksheet>
@@ -4264,125 +4319,143 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="18" customWidth="1"/>
-    <col min="2" max="3" width="28" customWidth="1"/>
+    <col min="2" max="2" width="18" customWidth="1"/>
+    <col min="3" max="4" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="14" t="s">
-        <v>5</v>
-      </c>
-      <c r="B1" s="14"/>
+    <row r="1" spans="1:4" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B1" s="14" t="s">
+        <v>4</v>
+      </c>
       <c r="C1" s="14"/>
-    </row>
-    <row r="2" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
+      <c r="D1" s="14"/>
+    </row>
+    <row r="2" spans="1:4" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A3" s="2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" s="2">
         <v>48</v>
       </c>
-      <c r="B3" s="8">
+      <c r="C3" s="8">
         <v>514</v>
       </c>
-      <c r="C3" s="3">
+      <c r="D3" s="3">
         <v>86</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A4" s="4">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B4" s="4">
         <v>96</v>
       </c>
-      <c r="B4" s="9">
+      <c r="C4" s="9">
         <v>1453</v>
       </c>
-      <c r="C4" s="5">
+      <c r="D4" s="5">
         <v>389</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A5" s="2">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="2">
         <v>144</v>
       </c>
-      <c r="B5" s="8">
+      <c r="C5" s="8">
         <v>3765</v>
       </c>
-      <c r="C5" s="3">
+      <c r="D5" s="3">
         <v>1147</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A6" s="4">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="4">
         <v>192</v>
       </c>
-      <c r="B6" s="9">
+      <c r="C6" s="9">
         <v>5970</v>
       </c>
-      <c r="C6" s="5">
+      <c r="D6" s="5">
         <v>2946</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A7" s="2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" s="2">
         <v>240</v>
       </c>
-      <c r="B7" s="8">
+      <c r="C7" s="8">
         <v>10922</v>
       </c>
-      <c r="C7" s="3">
+      <c r="D7" s="3">
         <v>6483</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A8" s="4">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="4">
         <v>288</v>
       </c>
-      <c r="B8" s="9">
+      <c r="C8" s="9">
         <v>17083</v>
       </c>
-      <c r="C8" s="5">
+      <c r="D8" s="5">
         <v>11449</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A9" s="2"/>
-      <c r="B9" s="3"/>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B9" s="2"/>
       <c r="C9" s="3"/>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A10" s="4"/>
-      <c r="B10" s="5"/>
+      <c r="D9" s="3"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B10" s="4"/>
       <c r="C10" s="5"/>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A11" s="2"/>
-      <c r="B11" s="3"/>
+      <c r="D10" s="5"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B11" s="2"/>
       <c r="C11" s="3"/>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A12" s="4"/>
-      <c r="B12" s="5"/>
+      <c r="D11" s="3"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B12" s="4"/>
       <c r="C12" s="5"/>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A13" s="2"/>
-      <c r="B13" s="3"/>
+      <c r="D12" s="5"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B13" s="2"/>
       <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="B1:D1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>